<commit_message>
restructuring for agile development for a more cohesive code base
</commit_message>
<xml_diff>
--- a/planning/QKD Admin.xlsx
+++ b/planning/QKD Admin.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7133c30a7a32802d/Documents/NCL/Year 3/QKD/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7133c30a7a32802d/Documents/NCL/Year 3/QKD/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="362" documentId="8_{C223F488-EF60-4955-8651-718FF70ED26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6056B6B0-E4C4-4E6A-8A97-0CAB23B61B95}"/>
+  <xr:revisionPtr revIDLastSave="371" documentId="8_{C223F488-EF60-4955-8651-718FF70ED26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{016B70AC-EEE2-4EE8-894F-EB023DC06D33}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{1D60F646-B254-4177-90BA-2D22A29CC258}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Lit Review" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="119">
   <si>
     <t>Week Beginning</t>
   </si>
@@ -385,7 +384,16 @@
     <t>poster pres</t>
   </si>
   <si>
-    <t>guide on engineering postersssh-keygen -t ed25519 -C "your_email@example.com"</t>
+    <t>QKD Key management systems overview</t>
+  </si>
+  <si>
+    <t>KMS paper</t>
+  </si>
+  <si>
+    <t>May be a useful evolution of the simulations</t>
+  </si>
+  <si>
+    <t>guide on engineering posters</t>
   </si>
 </sst>
 </file>
@@ -1866,10 +1874,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3147,18 +3151,30 @@
         <v>113</v>
       </c>
       <c r="F24" s="28" t="s">
+        <v>118</v>
+      </c>
+      <c r="G24" s="29"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="G24" s="29"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="27"/>
       <c r="B25" s="27"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="29"/>
+      <c r="C25" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="E25" s="59" t="s">
+        <v>116</v>
+      </c>
+      <c r="F25" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="G25" s="29" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="27"/>
@@ -3914,6 +3930,7 @@
     <hyperlink ref="E22" r:id="rId21" xr:uid="{9CC89986-CE00-431A-9DD4-A9495D2623A2}"/>
     <hyperlink ref="E23" r:id="rId22" xr:uid="{97DC5BB5-DD4D-4574-AAAE-73CA715FC8E9}"/>
     <hyperlink ref="E24" r:id="rId23" xr:uid="{4ABAD634-FD14-484A-A732-E29574983E3F}"/>
+    <hyperlink ref="E25" r:id="rId24" xr:uid="{D21A592D-0334-4D3B-A1F8-2ED4F5DDFFFA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
huge refactor, new system integration, and full project restructure
Combines four local commits into one clean commit, excluding large
asset folders (literature/, planning/, poster/) that exceeded git
size limits. Adds .gitignore to prevent these from being re-tracked.

Originally comprised:
- adding new literature and planning documents, for PRD for future developments
- ADMIN UPDATE: Updated QKD Admin spreadsheet with latest project details
- huge refactor, new system integration, and full project restructure
- system updated following refactor
</commit_message>
<xml_diff>
--- a/planning/QKD Admin.xlsx
+++ b/planning/QKD Admin.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7133c30a7a32802d/Documents/NCL/Year 3/QKD/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="371" documentId="8_{C223F488-EF60-4955-8651-718FF70ED26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{016B70AC-EEE2-4EE8-894F-EB023DC06D33}"/>
+  <xr:revisionPtr revIDLastSave="389" documentId="8_{C223F488-EF60-4955-8651-718FF70ED26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{705C466A-DB82-4A7A-92F0-A8AA846A1227}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{1D60F646-B254-4177-90BA-2D22A29CC258}"/>
+    <workbookView minimized="1" xWindow="30360" yWindow="1560" windowWidth="21600" windowHeight="11175" activeTab="1" xr2:uid="{1D60F646-B254-4177-90BA-2D22A29CC258}"/>
   </bookViews>
   <sheets>
     <sheet name="Timesheet" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="125">
   <si>
     <t>Week Beginning</t>
   </si>
@@ -96,9 +96,6 @@
     <t>Review of Algorthims</t>
   </si>
   <si>
-    <t>Useful breakdown on current systems, limitations, and potential advancements</t>
-  </si>
-  <si>
     <t>Kairostay: QKD implementation/ cyber nerd</t>
   </si>
   <si>
@@ -394,6 +391,27 @@
   </si>
   <si>
     <t>guide on engineering posters</t>
+  </si>
+  <si>
+    <t>e91 implementatio</t>
+  </si>
+  <si>
+    <t>paper</t>
+  </si>
+  <si>
+    <t>scope</t>
+  </si>
+  <si>
+    <t>e91 implmentation</t>
+  </si>
+  <si>
+    <t>nice visuals, look to implement something similar</t>
+  </si>
+  <si>
+    <t>e91 guide</t>
+  </si>
+  <si>
+    <t>USE FOR MODELLING SCENARIOS, vbery good domain specific examples &amp; roadmap directional attention</t>
   </si>
 </sst>
 </file>
@@ -764,7 +782,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="10" xfId="2" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
@@ -1066,55 +1084,55 @@
                   <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>48</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1874,6 +1892,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2192,12 +2214,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80F9B144-5C3E-47EA-AFD9-2007492993E3}">
   <dimension ref="D2:G37"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="7" width="16.6328125" customWidth="1"/>
+    <col min="4" max="7" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="4:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E2" s="4" t="s">
         <v>0</v>
       </c>
@@ -2208,7 +2230,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="4:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="4:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="E3" s="6">
         <v>45929</v>
       </c>
@@ -2220,7 +2242,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E4" s="3">
         <v>45936</v>
       </c>
@@ -2232,7 +2254,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E5" s="3">
         <v>45943</v>
       </c>
@@ -2244,7 +2266,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E6" s="3">
         <v>45950</v>
       </c>
@@ -2256,7 +2278,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D7" s="14" t="s">
         <v>3</v>
       </c>
@@ -2271,7 +2293,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E8" s="3">
         <v>45964</v>
       </c>
@@ -2283,7 +2305,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E9" s="3">
         <v>45971</v>
       </c>
@@ -2295,7 +2317,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E10" s="3">
         <v>45978</v>
       </c>
@@ -2307,7 +2329,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E11" s="3">
         <v>45985</v>
       </c>
@@ -2319,7 +2341,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E12" s="3">
         <v>45992</v>
       </c>
@@ -2331,7 +2353,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E13" s="3">
         <v>45999</v>
       </c>
@@ -2343,7 +2365,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E14" s="3">
         <v>46006</v>
       </c>
@@ -2355,7 +2377,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E15" s="3">
         <v>46013</v>
       </c>
@@ -2367,7 +2389,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E16" s="3">
         <v>46020</v>
       </c>
@@ -2379,7 +2401,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E17" s="3">
         <v>46027</v>
       </c>
@@ -2391,7 +2413,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E18" s="3">
         <v>46034</v>
       </c>
@@ -2403,7 +2425,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E19" s="3">
         <v>46041</v>
       </c>
@@ -2415,19 +2437,19 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="4:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E20" s="3">
         <v>46048</v>
       </c>
       <c r="F20" s="10">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G20" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E21" s="3">
         <v>46055</v>
       </c>
@@ -2436,10 +2458,10 @@
       </c>
       <c r="G21" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="22" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D22" s="18" t="s">
         <v>4</v>
       </c>
@@ -2451,10 +2473,10 @@
       </c>
       <c r="G22" s="17">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="23" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E23" s="3">
         <v>46069</v>
       </c>
@@ -2463,10 +2485,10 @@
       </c>
       <c r="G23" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E24" s="3">
         <v>46076</v>
       </c>
@@ -2475,10 +2497,10 @@
       </c>
       <c r="G24" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="25" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E25" s="3">
         <v>46083</v>
       </c>
@@ -2487,10 +2509,10 @@
       </c>
       <c r="G25" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="26" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E26" s="3">
         <v>46090</v>
       </c>
@@ -2499,10 +2521,10 @@
       </c>
       <c r="G26" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E27" s="3">
         <v>46097</v>
       </c>
@@ -2511,10 +2533,10 @@
       </c>
       <c r="G27" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="28" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E28" s="3">
         <v>46104</v>
       </c>
@@ -2523,10 +2545,10 @@
       </c>
       <c r="G28" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="29" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E29" s="3">
         <v>46111</v>
       </c>
@@ -2535,10 +2557,10 @@
       </c>
       <c r="G29" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="30" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="30" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E30" s="3">
         <v>46118</v>
       </c>
@@ -2547,10 +2569,10 @@
       </c>
       <c r="G30" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="31" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E31" s="3">
         <v>46125</v>
       </c>
@@ -2559,10 +2581,10 @@
       </c>
       <c r="G31" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="32" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E32" s="3">
         <v>46132</v>
       </c>
@@ -2571,10 +2593,10 @@
       </c>
       <c r="G32" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="33" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D33" s="19" t="s">
         <v>5</v>
       </c>
@@ -2586,10 +2608,10 @@
       </c>
       <c r="G33" s="22">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="34" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E34" s="3">
         <v>46146</v>
       </c>
@@ -2598,10 +2620,10 @@
       </c>
       <c r="G34" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="35" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D35" s="23" t="s">
         <v>6</v>
       </c>
@@ -2613,10 +2635,10 @@
       </c>
       <c r="G35" s="26">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="36" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E36" s="3">
         <v>46160</v>
       </c>
@@ -2625,10 +2647,10 @@
       </c>
       <c r="G36" s="2">
         <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="37" spans="4:7" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" spans="4:7" x14ac:dyDescent="0.25">
       <c r="E37" s="1"/>
     </row>
   </sheetData>
@@ -2640,29 +2662,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4974D2B-3CED-442F-8F5D-4F7E9530009D}">
   <dimension ref="A1:G106"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
-    <col min="2" max="2" width="9.08984375" customWidth="1"/>
-    <col min="3" max="3" width="20.6328125" customWidth="1"/>
-    <col min="4" max="4" width="25.453125" customWidth="1"/>
-    <col min="5" max="5" width="20.6328125" customWidth="1"/>
-    <col min="6" max="6" width="44.90625" customWidth="1"/>
-    <col min="7" max="7" width="200.6328125" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="25.42578125" customWidth="1"/>
+    <col min="5" max="5" width="20.5703125" customWidth="1"/>
+    <col min="6" max="6" width="44.85546875" customWidth="1"/>
+    <col min="7" max="7" width="200.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="30" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="30" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C1" s="31" t="s">
         <v>8</v>
       </c>
       <c r="D1" s="31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E1" s="31" t="s">
         <v>9</v>
@@ -2674,7 +2696,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="37" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" s="37" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
         <v>15</v>
       </c>
@@ -2683,10 +2705,10 @@
         <v>12</v>
       </c>
       <c r="D2" s="34" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F2" s="34" t="s">
         <v>13</v>
@@ -2695,497 +2717,509 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="58"/>
+      <c r="B3" s="57"/>
       <c r="C3" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D3" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E3" s="40" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F3" s="39" t="s">
         <v>18</v>
       </c>
       <c r="G3" s="41" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="50" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="46" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" s="50" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="46" t="s">
-        <v>20</v>
       </c>
       <c r="B4" s="58"/>
       <c r="C4" s="47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D4" s="47" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E4" s="48" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="49" t="s">
+    </row>
+    <row r="5" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="42" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="42" t="s">
-        <v>23</v>
       </c>
       <c r="B5" s="58"/>
       <c r="C5" s="43" t="s">
         <v>17</v>
       </c>
       <c r="D5" s="43" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F5" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="45" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="50" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="45" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" s="50" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="46" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="58"/>
+      <c r="B6" s="57"/>
       <c r="C6" s="47" t="s">
         <v>17</v>
       </c>
       <c r="D6" s="47" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E6" s="48" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F6" s="47" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G6" s="49" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="38" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="38" t="s">
-        <v>34</v>
       </c>
       <c r="B7" s="58"/>
       <c r="C7" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D7" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E7" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="39" t="s">
+      <c r="G7" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="G7" s="41" t="s">
+    </row>
+    <row r="8" spans="1:7" s="56" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="52" t="s">
         <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="56" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="52" t="s">
-        <v>38</v>
       </c>
       <c r="B8" s="57"/>
       <c r="C8" s="53" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="53" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E8" s="54" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="53" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="53" t="s">
+      <c r="G8" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="G8" s="55" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" s="58"/>
+        <v>42</v>
+      </c>
+      <c r="B9" s="57"/>
       <c r="C9" s="43" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E9" s="44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F9" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="45" t="s">
         <v>44</v>
       </c>
-      <c r="G9" s="45" t="s">
+    </row>
+    <row r="10" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="38" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="38" t="s">
-        <v>46</v>
       </c>
       <c r="B10" s="57"/>
       <c r="C10" s="39" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E10" s="40" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="F10" s="39" t="s">
+      <c r="G10" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="G10" s="41" t="s">
+    </row>
+    <row r="11" spans="1:7" s="56" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="52" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" s="56" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="52" t="s">
-        <v>50</v>
       </c>
       <c r="B11" s="57"/>
       <c r="C11" s="53" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="53" t="s">
+        <v>96</v>
+      </c>
+      <c r="E11" s="54" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="53" t="s">
-        <v>97</v>
-      </c>
-      <c r="E11" s="54" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" s="53" t="s">
+      <c r="G11" s="55" t="s">
         <v>52</v>
       </c>
-      <c r="G11" s="55" t="s">
+    </row>
+    <row r="12" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="38" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="38" t="s">
-        <v>54</v>
       </c>
       <c r="B12" s="58"/>
       <c r="C12" s="39" t="s">
         <v>17</v>
       </c>
       <c r="D12" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E12" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="39" t="s">
         <v>55</v>
       </c>
-      <c r="F12" s="39" t="s">
+      <c r="G12" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="G12" s="41" t="s">
+    </row>
+    <row r="13" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="38" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="38" t="s">
-        <v>58</v>
       </c>
       <c r="B13" s="58"/>
       <c r="C13" s="39" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="E13" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="39" t="s">
-        <v>94</v>
-      </c>
-      <c r="E13" s="40" t="s">
+      <c r="F13" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="F13" s="39" t="s">
+      <c r="G13" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="G13" s="41" t="s">
+    </row>
+    <row r="14" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="42" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="42" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="58"/>
+      <c r="B14" s="57"/>
       <c r="C14" s="43" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E14" s="51" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="G14" s="45" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="42" t="s">
         <v>64</v>
-      </c>
-      <c r="F14" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="G14" s="45" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="42" t="s">
-        <v>65</v>
       </c>
       <c r="B15" s="58"/>
       <c r="C15" s="43" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E15" s="44" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F15" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="G15" s="45" t="s">
         <v>69</v>
       </c>
-      <c r="G15" s="45" t="s">
+    </row>
+    <row r="16" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="42" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="42" t="s">
-        <v>71</v>
       </c>
       <c r="B16" s="57"/>
       <c r="C16" s="43" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="43" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E16" s="44" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="43" t="s">
         <v>72</v>
       </c>
-      <c r="F16" s="43" t="s">
+      <c r="G16" s="45" t="s">
         <v>73</v>
       </c>
-      <c r="G16" s="45" t="s">
+    </row>
+    <row r="17" spans="1:7" s="50" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="46" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" s="50" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="46" t="s">
-        <v>75</v>
       </c>
       <c r="B17" s="58"/>
       <c r="C17" s="47" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="47" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E17" s="48" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" s="47" t="s">
         <v>76</v>
       </c>
-      <c r="F17" s="47" t="s">
+      <c r="G17" s="49" t="s">
         <v>77</v>
       </c>
-      <c r="G17" s="49" t="s">
+    </row>
+    <row r="18" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="38" t="s">
         <v>78</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="38" t="s">
-        <v>79</v>
       </c>
       <c r="B18" s="58"/>
       <c r="C18" s="39" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E18" s="40" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="39" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="39" t="s">
+      <c r="G18" s="41" t="s">
         <v>81</v>
       </c>
-      <c r="G18" s="41" t="s">
+    </row>
+    <row r="19" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="38" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="38" t="s">
-        <v>83</v>
       </c>
       <c r="B19" s="58"/>
       <c r="C19" s="39" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E19" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" s="39" t="s">
         <v>84</v>
       </c>
-      <c r="F19" s="39" t="s">
+      <c r="G19" s="41" t="s">
         <v>85</v>
       </c>
-      <c r="G19" s="41" t="s">
+    </row>
+    <row r="20" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="42" t="s">
         <v>86</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" s="37" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="42" t="s">
-        <v>87</v>
       </c>
       <c r="B20" s="58"/>
       <c r="C20" s="43" t="s">
         <v>12</v>
       </c>
       <c r="D20" s="43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E20" s="44" t="s">
+        <v>87</v>
+      </c>
+      <c r="F20" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="F20" s="43" t="s">
+      <c r="G20" s="45" t="s">
         <v>89</v>
       </c>
-      <c r="G20" s="45" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="38" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B21" s="57"/>
       <c r="C21" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="E21" s="40" t="s">
         <v>99</v>
       </c>
-      <c r="D21" s="39" t="s">
-        <v>94</v>
-      </c>
-      <c r="E21" s="40" t="s">
+      <c r="F21" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="F21" s="39" t="s">
+      <c r="G21" s="41" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="G21" s="41" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="38" t="s">
-        <v>102</v>
-      </c>
-      <c r="B22" s="58"/>
+      <c r="B22" s="57"/>
       <c r="C22" s="39" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E22" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="F22" s="39" t="s">
         <v>103</v>
       </c>
-      <c r="F22" s="39" t="s">
+      <c r="G22" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="G22" s="41" t="s">
+    </row>
+    <row r="23" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="38" t="s">
         <v>105</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="38" t="s">
-        <v>106</v>
       </c>
       <c r="B23" s="57"/>
       <c r="C23" s="39" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E23" s="40" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="F23" s="39" t="s">
+      <c r="G23" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="G23" s="41" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="27" t="s">
+    </row>
+    <row r="24" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="B24" s="59"/>
+      <c r="C24" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="28" t="s">
+      <c r="D24" s="39" t="s">
         <v>113</v>
       </c>
-      <c r="D24" s="28" t="s">
+      <c r="E24" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="F24" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="G24" s="41"/>
+    </row>
+    <row r="25" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="38" t="s">
         <v>114</v>
       </c>
-      <c r="E24" s="59" t="s">
-        <v>113</v>
-      </c>
-      <c r="F24" s="28" t="s">
+      <c r="B25" s="59"/>
+      <c r="C25" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="E25" s="40" t="s">
+        <v>115</v>
+      </c>
+      <c r="F25" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="G25" s="41" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="G24" s="29"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="27" t="s">
-        <v>115</v>
-      </c>
-      <c r="B25" s="27"/>
-      <c r="C25" s="28" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="E25" s="59" t="s">
-        <v>116</v>
-      </c>
-      <c r="F25" s="28" t="s">
-        <v>116</v>
-      </c>
-      <c r="G25" s="29" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="27"/>
-      <c r="B26" s="27"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="29"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B26" s="59"/>
+      <c r="C26" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="E26" s="40" t="s">
+        <v>123</v>
+      </c>
+      <c r="F26" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="G26" s="41" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="27"/>
       <c r="B27" s="27"/>
       <c r="C27" s="28"/>
@@ -3194,7 +3228,7 @@
       <c r="F27" s="28"/>
       <c r="G27" s="29"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="27"/>
       <c r="B28" s="27"/>
       <c r="C28" s="28"/>
@@ -3203,7 +3237,7 @@
       <c r="F28" s="28"/>
       <c r="G28" s="29"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="27"/>
       <c r="B29" s="27"/>
       <c r="C29" s="28"/>
@@ -3212,7 +3246,7 @@
       <c r="F29" s="28"/>
       <c r="G29" s="29"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="27"/>
       <c r="B30" s="27"/>
       <c r="C30" s="28"/>
@@ -3221,7 +3255,7 @@
       <c r="F30" s="28"/>
       <c r="G30" s="29"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="27"/>
       <c r="B31" s="27"/>
       <c r="C31" s="28"/>
@@ -3230,7 +3264,7 @@
       <c r="F31" s="28"/>
       <c r="G31" s="29"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="27"/>
       <c r="B32" s="27"/>
       <c r="C32" s="28"/>
@@ -3239,7 +3273,7 @@
       <c r="F32" s="28"/>
       <c r="G32" s="29"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="27"/>
       <c r="B33" s="27"/>
       <c r="C33" s="28"/>
@@ -3248,7 +3282,7 @@
       <c r="F33" s="28"/>
       <c r="G33" s="29"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="27"/>
       <c r="B34" s="27"/>
       <c r="C34" s="28"/>
@@ -3257,7 +3291,7 @@
       <c r="F34" s="28"/>
       <c r="G34" s="29"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="27"/>
       <c r="B35" s="27"/>
       <c r="C35" s="28"/>
@@ -3266,7 +3300,7 @@
       <c r="F35" s="28"/>
       <c r="G35" s="29"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="27"/>
       <c r="B36" s="27"/>
       <c r="C36" s="28"/>
@@ -3275,7 +3309,7 @@
       <c r="F36" s="28"/>
       <c r="G36" s="29"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="27"/>
       <c r="B37" s="27"/>
       <c r="C37" s="28"/>
@@ -3284,7 +3318,7 @@
       <c r="F37" s="28"/>
       <c r="G37" s="29"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="27"/>
       <c r="B38" s="27"/>
       <c r="C38" s="28"/>
@@ -3293,7 +3327,7 @@
       <c r="F38" s="28"/>
       <c r="G38" s="29"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="27"/>
       <c r="B39" s="27"/>
       <c r="C39" s="28"/>
@@ -3302,7 +3336,7 @@
       <c r="F39" s="28"/>
       <c r="G39" s="29"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="27"/>
       <c r="B40" s="27"/>
       <c r="C40" s="28"/>
@@ -3311,7 +3345,7 @@
       <c r="F40" s="28"/>
       <c r="G40" s="29"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="27"/>
       <c r="B41" s="27"/>
       <c r="C41" s="28"/>
@@ -3320,7 +3354,7 @@
       <c r="F41" s="28"/>
       <c r="G41" s="29"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="27"/>
       <c r="B42" s="27"/>
       <c r="C42" s="28"/>
@@ -3329,7 +3363,7 @@
       <c r="F42" s="28"/>
       <c r="G42" s="29"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="27"/>
       <c r="B43" s="27"/>
       <c r="C43" s="28"/>
@@ -3338,7 +3372,7 @@
       <c r="F43" s="28"/>
       <c r="G43" s="29"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="27"/>
       <c r="B44" s="27"/>
       <c r="C44" s="28"/>
@@ -3347,7 +3381,7 @@
       <c r="F44" s="28"/>
       <c r="G44" s="29"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="27"/>
       <c r="B45" s="27"/>
       <c r="C45" s="28"/>
@@ -3356,7 +3390,7 @@
       <c r="F45" s="28"/>
       <c r="G45" s="29"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="27"/>
       <c r="B46" s="27"/>
       <c r="C46" s="28"/>
@@ -3365,7 +3399,7 @@
       <c r="F46" s="28"/>
       <c r="G46" s="29"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="27"/>
       <c r="B47" s="27"/>
       <c r="C47" s="28"/>
@@ -3374,7 +3408,7 @@
       <c r="F47" s="28"/>
       <c r="G47" s="29"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="27"/>
       <c r="B48" s="27"/>
       <c r="C48" s="28"/>
@@ -3383,7 +3417,7 @@
       <c r="F48" s="28"/>
       <c r="G48" s="29"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="27"/>
       <c r="B49" s="27"/>
       <c r="C49" s="28"/>
@@ -3392,7 +3426,7 @@
       <c r="F49" s="28"/>
       <c r="G49" s="29"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="27"/>
       <c r="B50" s="27"/>
       <c r="C50" s="28"/>
@@ -3401,7 +3435,7 @@
       <c r="F50" s="28"/>
       <c r="G50" s="29"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="27"/>
       <c r="B51" s="27"/>
       <c r="C51" s="28"/>
@@ -3410,7 +3444,7 @@
       <c r="F51" s="28"/>
       <c r="G51" s="29"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="27"/>
       <c r="B52" s="27"/>
       <c r="C52" s="28"/>
@@ -3419,7 +3453,7 @@
       <c r="F52" s="28"/>
       <c r="G52" s="29"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="27"/>
       <c r="B53" s="27"/>
       <c r="C53" s="28"/>
@@ -3428,7 +3462,7 @@
       <c r="F53" s="28"/>
       <c r="G53" s="29"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="27"/>
       <c r="B54" s="27"/>
       <c r="C54" s="28"/>
@@ -3437,7 +3471,7 @@
       <c r="F54" s="28"/>
       <c r="G54" s="29"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="27"/>
       <c r="B55" s="27"/>
       <c r="C55" s="28"/>
@@ -3446,7 +3480,7 @@
       <c r="F55" s="28"/>
       <c r="G55" s="29"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="27"/>
       <c r="B56" s="27"/>
       <c r="C56" s="28"/>
@@ -3455,7 +3489,7 @@
       <c r="F56" s="28"/>
       <c r="G56" s="29"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="27"/>
       <c r="B57" s="27"/>
       <c r="C57" s="28"/>
@@ -3464,7 +3498,7 @@
       <c r="F57" s="28"/>
       <c r="G57" s="29"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="27"/>
       <c r="B58" s="27"/>
       <c r="C58" s="28"/>
@@ -3473,7 +3507,7 @@
       <c r="F58" s="28"/>
       <c r="G58" s="29"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="27"/>
       <c r="B59" s="27"/>
       <c r="C59" s="28"/>
@@ -3482,7 +3516,7 @@
       <c r="F59" s="28"/>
       <c r="G59" s="29"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="27"/>
       <c r="B60" s="27"/>
       <c r="C60" s="28"/>
@@ -3491,7 +3525,7 @@
       <c r="F60" s="28"/>
       <c r="G60" s="29"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="27"/>
       <c r="B61" s="27"/>
       <c r="C61" s="28"/>
@@ -3500,7 +3534,7 @@
       <c r="F61" s="28"/>
       <c r="G61" s="29"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="27"/>
       <c r="B62" s="27"/>
       <c r="C62" s="28"/>
@@ -3509,7 +3543,7 @@
       <c r="F62" s="28"/>
       <c r="G62" s="29"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="27"/>
       <c r="B63" s="27"/>
       <c r="C63" s="28"/>
@@ -3518,7 +3552,7 @@
       <c r="F63" s="28"/>
       <c r="G63" s="29"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="27"/>
       <c r="B64" s="27"/>
       <c r="C64" s="28"/>
@@ -3527,7 +3561,7 @@
       <c r="F64" s="28"/>
       <c r="G64" s="29"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="27"/>
       <c r="B65" s="27"/>
       <c r="C65" s="28"/>
@@ -3536,7 +3570,7 @@
       <c r="F65" s="28"/>
       <c r="G65" s="29"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="27"/>
       <c r="B66" s="27"/>
       <c r="C66" s="28"/>
@@ -3545,7 +3579,7 @@
       <c r="F66" s="28"/>
       <c r="G66" s="29"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="27"/>
       <c r="B67" s="27"/>
       <c r="C67" s="28"/>
@@ -3554,7 +3588,7 @@
       <c r="F67" s="28"/>
       <c r="G67" s="29"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="27"/>
       <c r="B68" s="27"/>
       <c r="C68" s="28"/>
@@ -3563,7 +3597,7 @@
       <c r="F68" s="28"/>
       <c r="G68" s="29"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="27"/>
       <c r="B69" s="27"/>
       <c r="C69" s="28"/>
@@ -3572,7 +3606,7 @@
       <c r="F69" s="28"/>
       <c r="G69" s="29"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="27"/>
       <c r="B70" s="27"/>
       <c r="C70" s="28"/>
@@ -3581,7 +3615,7 @@
       <c r="F70" s="28"/>
       <c r="G70" s="29"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="27"/>
       <c r="B71" s="27"/>
       <c r="C71" s="28"/>
@@ -3590,7 +3624,7 @@
       <c r="F71" s="28"/>
       <c r="G71" s="29"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="27"/>
       <c r="B72" s="27"/>
       <c r="C72" s="28"/>
@@ -3599,7 +3633,7 @@
       <c r="F72" s="28"/>
       <c r="G72" s="29"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="27"/>
       <c r="B73" s="27"/>
       <c r="C73" s="28"/>
@@ -3608,7 +3642,7 @@
       <c r="F73" s="28"/>
       <c r="G73" s="29"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="27"/>
       <c r="B74" s="27"/>
       <c r="C74" s="28"/>
@@ -3617,7 +3651,7 @@
       <c r="F74" s="28"/>
       <c r="G74" s="29"/>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="27"/>
       <c r="B75" s="27"/>
       <c r="C75" s="28"/>
@@ -3626,7 +3660,7 @@
       <c r="F75" s="28"/>
       <c r="G75" s="29"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="27"/>
       <c r="B76" s="27"/>
       <c r="C76" s="28"/>
@@ -3635,7 +3669,7 @@
       <c r="F76" s="28"/>
       <c r="G76" s="29"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="27"/>
       <c r="B77" s="27"/>
       <c r="C77" s="28"/>
@@ -3644,7 +3678,7 @@
       <c r="F77" s="28"/>
       <c r="G77" s="29"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="27"/>
       <c r="B78" s="27"/>
       <c r="C78" s="28"/>
@@ -3653,7 +3687,7 @@
       <c r="F78" s="28"/>
       <c r="G78" s="29"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="27"/>
       <c r="B79" s="27"/>
       <c r="C79" s="28"/>
@@ -3662,7 +3696,7 @@
       <c r="F79" s="28"/>
       <c r="G79" s="29"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="27"/>
       <c r="B80" s="27"/>
       <c r="C80" s="28"/>
@@ -3671,7 +3705,7 @@
       <c r="F80" s="28"/>
       <c r="G80" s="29"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="27"/>
       <c r="B81" s="27"/>
       <c r="C81" s="28"/>
@@ -3680,7 +3714,7 @@
       <c r="F81" s="28"/>
       <c r="G81" s="29"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="27"/>
       <c r="B82" s="27"/>
       <c r="C82" s="28"/>
@@ -3689,7 +3723,7 @@
       <c r="F82" s="28"/>
       <c r="G82" s="29"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="27"/>
       <c r="B83" s="27"/>
       <c r="C83" s="28"/>
@@ -3698,7 +3732,7 @@
       <c r="F83" s="28"/>
       <c r="G83" s="29"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="27"/>
       <c r="B84" s="27"/>
       <c r="C84" s="28"/>
@@ -3707,7 +3741,7 @@
       <c r="F84" s="28"/>
       <c r="G84" s="29"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="27"/>
       <c r="B85" s="27"/>
       <c r="C85" s="28"/>
@@ -3716,7 +3750,7 @@
       <c r="F85" s="28"/>
       <c r="G85" s="29"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="27"/>
       <c r="B86" s="27"/>
       <c r="C86" s="28"/>
@@ -3725,7 +3759,7 @@
       <c r="F86" s="28"/>
       <c r="G86" s="29"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="27"/>
       <c r="B87" s="27"/>
       <c r="C87" s="28"/>
@@ -3734,7 +3768,7 @@
       <c r="F87" s="28"/>
       <c r="G87" s="29"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="27"/>
       <c r="B88" s="27"/>
       <c r="C88" s="28"/>
@@ -3743,7 +3777,7 @@
       <c r="F88" s="28"/>
       <c r="G88" s="29"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="27"/>
       <c r="B89" s="27"/>
       <c r="C89" s="28"/>
@@ -3752,7 +3786,7 @@
       <c r="F89" s="28"/>
       <c r="G89" s="29"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="27"/>
       <c r="B90" s="27"/>
       <c r="C90" s="28"/>
@@ -3761,7 +3795,7 @@
       <c r="F90" s="28"/>
       <c r="G90" s="29"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="27"/>
       <c r="B91" s="27"/>
       <c r="C91" s="28"/>
@@ -3770,7 +3804,7 @@
       <c r="F91" s="28"/>
       <c r="G91" s="29"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="27"/>
       <c r="B92" s="27"/>
       <c r="C92" s="28"/>
@@ -3779,7 +3813,7 @@
       <c r="F92" s="28"/>
       <c r="G92" s="29"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="27"/>
       <c r="B93" s="27"/>
       <c r="C93" s="28"/>
@@ -3788,7 +3822,7 @@
       <c r="F93" s="28"/>
       <c r="G93" s="29"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="27"/>
       <c r="B94" s="27"/>
       <c r="C94" s="28"/>
@@ -3797,7 +3831,7 @@
       <c r="F94" s="28"/>
       <c r="G94" s="29"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="27"/>
       <c r="B95" s="27"/>
       <c r="C95" s="28"/>
@@ -3806,7 +3840,7 @@
       <c r="F95" s="28"/>
       <c r="G95" s="29"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="27"/>
       <c r="B96" s="27"/>
       <c r="C96" s="28"/>
@@ -3815,7 +3849,7 @@
       <c r="F96" s="28"/>
       <c r="G96" s="29"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="27"/>
       <c r="B97" s="27"/>
       <c r="C97" s="28"/>
@@ -3824,7 +3858,7 @@
       <c r="F97" s="28"/>
       <c r="G97" s="29"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="27"/>
       <c r="B98" s="27"/>
       <c r="C98" s="28"/>
@@ -3833,7 +3867,7 @@
       <c r="F98" s="28"/>
       <c r="G98" s="29"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="27"/>
       <c r="B99" s="27"/>
       <c r="C99" s="28"/>
@@ -3842,7 +3876,7 @@
       <c r="F99" s="28"/>
       <c r="G99" s="29"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="27"/>
       <c r="B100" s="27"/>
       <c r="C100" s="28"/>
@@ -3851,7 +3885,7 @@
       <c r="F100" s="28"/>
       <c r="G100" s="29"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="27"/>
       <c r="B101" s="27"/>
       <c r="C101" s="28"/>
@@ -3860,7 +3894,7 @@
       <c r="F101" s="28"/>
       <c r="G101" s="29"/>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="27"/>
       <c r="B102" s="27"/>
       <c r="C102" s="28"/>
@@ -3869,7 +3903,7 @@
       <c r="F102" s="28"/>
       <c r="G102" s="29"/>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="27"/>
       <c r="B103" s="27"/>
       <c r="C103" s="28"/>
@@ -3878,7 +3912,7 @@
       <c r="F103" s="28"/>
       <c r="G103" s="29"/>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="27"/>
       <c r="B104" s="27"/>
       <c r="C104" s="28"/>
@@ -3887,7 +3921,7 @@
       <c r="F104" s="28"/>
       <c r="G104" s="29"/>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="27"/>
       <c r="B105" s="27"/>
       <c r="C105" s="28"/>
@@ -3896,7 +3930,7 @@
       <c r="F105" s="28"/>
       <c r="G105" s="29"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="27"/>
       <c r="B106" s="27"/>
       <c r="C106" s="28"/>
@@ -3931,6 +3965,7 @@
     <hyperlink ref="E23" r:id="rId22" xr:uid="{97DC5BB5-DD4D-4574-AAAE-73CA715FC8E9}"/>
     <hyperlink ref="E24" r:id="rId23" xr:uid="{4ABAD634-FD14-484A-A732-E29574983E3F}"/>
     <hyperlink ref="E25" r:id="rId24" xr:uid="{D21A592D-0334-4D3B-A1F8-2ED4F5DDFFFA}"/>
+    <hyperlink ref="E26" r:id="rId25" xr:uid="{C745BC45-2A05-4987-8D50-BF85A9863A49}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>